<commit_message>
parallel execution and logging
</commit_message>
<xml_diff>
--- a/testData/OrangeHRMData.xlsx
+++ b/testData/OrangeHRMData.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Username</t>
   </si>
@@ -58,51 +58,6 @@
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>Vishnu</t>
-  </si>
-  <si>
-    <t>Vardhan</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>Hari</t>
-  </si>
-  <si>
-    <t>Charan</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>Sai</t>
-  </si>
-  <si>
-    <t>Sudharsan</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>Gopi</t>
-  </si>
-  <si>
-    <t>Chand</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>Shyam</t>
-  </si>
-  <si>
-    <t>Karan</t>
-  </si>
-  <si>
-    <t>R</t>
   </si>
 </sst>
 </file>
@@ -1283,8 +1238,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="2"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14.2222222222222" customWidth="1"/>
     <col min="2" max="2" width="11.4444444444444" customWidth="1"/>
@@ -1313,61 +1268,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>